<commit_message>
Atualiza dados do Smart Stock
</commit_message>
<xml_diff>
--- a/data-source/compras.xlsx
+++ b/data-source/compras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/prompt-smart-stock-sight (4) (1)antig/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_A326C178CB385EDFDA183B5B29A248968F540666" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFF126C9-B235-49A7-8439-BB89EF408E57}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="11_A326C178CB385EDFDA183B5B29A248968F540666" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4B0F912-A71B-437D-B77B-F72843E93EEB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="30">
   <si>
     <t>Núm.OC</t>
   </si>
@@ -76,9 +76,6 @@
     <t>SM3</t>
   </si>
   <si>
-    <t>NAPA METAL CHARM PRATA - PU 0.9MM</t>
-  </si>
-  <si>
     <t>NAPA BARI BEGE - PU 0.7MM</t>
   </si>
   <si>
@@ -94,15 +91,6 @@
     <t>NAPA BARI CAFE - PU 0.7MM</t>
   </si>
   <si>
-    <t>HELSINKI CAFE - 1.2MM</t>
-  </si>
-  <si>
-    <t>NAPA BARI BRANCO - PU 0.7MM</t>
-  </si>
-  <si>
-    <t>NAPA METAL CHARM PRETO - PU 0.9MM</t>
-  </si>
-  <si>
     <t>NAPA MADRID PRETO - PU 0.9MM</t>
   </si>
   <si>
@@ -122,6 +110,9 @@
   </si>
   <si>
     <t>NAPA METAL LYON OURO LIGHT - PU 0.9MM</t>
+  </si>
+  <si>
+    <t>NAPA METAL LYON PRATA - PU 0.9MM</t>
   </si>
 </sst>
 </file>
@@ -130,10 +121,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[Blue]###########0;[Red]\-###########0"/>
-    <numFmt numFmtId="166" formatCode="[Blue]###,###,###,##0.000;[Red]\-###,###,###,##0.000"/>
-    <numFmt numFmtId="167" formatCode="[Blue]###,###,###,##0.0000;[Red]\-###,###,###,##0.0000"/>
+    <numFmt numFmtId="165" formatCode="[Blue]###,###,###,##0.000;[Red]\-###,###,###,##0.000"/>
+    <numFmt numFmtId="166" formatCode="[Blue]###,###,###,##0.0000;[Red]\-###,###,###,##0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -146,6 +137,12 @@
       <sz val="11"/>
       <color rgb="FF800000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -194,8 +191,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -533,7 +530,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" customWidth="1"/>
@@ -598,7 +595,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="B2" s="2">
         <v>162</v>
@@ -607,10 +604,10 @@
         <v>14</v>
       </c>
       <c r="D2" s="4">
-        <v>46156</v>
+        <v>46183</v>
       </c>
       <c r="E2" s="2">
-        <v>20102</v>
+        <v>20000</v>
       </c>
       <c r="F2" s="2">
         <v>39</v>
@@ -619,22 +616,22 @@
         <v>40</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I2" s="5">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="J2" s="5">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="K2" s="6">
-        <v>2.08</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="L2" s="4">
-        <v>46187</v>
+        <v>46275</v>
       </c>
       <c r="M2" s="4">
-        <v>46187</v>
+        <v>46275</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>16</v>
@@ -642,7 +639,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="B3" s="2">
         <v>162</v>
@@ -651,10 +648,10 @@
         <v>14</v>
       </c>
       <c r="D3" s="4">
-        <v>46156</v>
+        <v>46183</v>
       </c>
       <c r="E3" s="2">
-        <v>20103</v>
+        <v>20011</v>
       </c>
       <c r="F3" s="2">
         <v>39</v>
@@ -663,22 +660,22 @@
         <v>40</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="I3" s="5">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="J3" s="5">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="K3" s="6">
-        <v>2.08</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="L3" s="4">
-        <v>46187</v>
+        <v>46275</v>
       </c>
       <c r="M3" s="4">
-        <v>46187</v>
+        <v>46275</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>16</v>
@@ -686,7 +683,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="B4" s="2">
         <v>162</v>
@@ -695,10 +692,10 @@
         <v>14</v>
       </c>
       <c r="D4" s="4">
-        <v>46156</v>
+        <v>46189</v>
       </c>
       <c r="E4" s="2">
-        <v>20104</v>
+        <v>20034</v>
       </c>
       <c r="F4" s="2">
         <v>39</v>
@@ -707,22 +704,22 @@
         <v>40</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" s="5">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="J4" s="5">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="K4" s="6">
         <v>1.32</v>
       </c>
       <c r="L4" s="4">
-        <v>46187</v>
+        <v>46281</v>
       </c>
       <c r="M4" s="4">
-        <v>46187</v>
+        <v>46281</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>16</v>
@@ -730,7 +727,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="B5" s="2">
         <v>162</v>
@@ -739,10 +736,10 @@
         <v>14</v>
       </c>
       <c r="D5" s="4">
-        <v>46156</v>
+        <v>46189</v>
       </c>
       <c r="E5" s="2">
-        <v>20105</v>
+        <v>20082</v>
       </c>
       <c r="F5" s="2">
         <v>39</v>
@@ -751,22 +748,22 @@
         <v>40</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I5" s="5">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="J5" s="5">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="K5" s="6">
         <v>1.32</v>
       </c>
       <c r="L5" s="4">
-        <v>46187</v>
+        <v>46281</v>
       </c>
       <c r="M5" s="4">
-        <v>46187</v>
+        <v>46281</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>16</v>
@@ -774,7 +771,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="B6" s="2">
         <v>162</v>
@@ -783,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="D6" s="4">
-        <v>46176</v>
+        <v>46189</v>
       </c>
       <c r="E6" s="2">
-        <v>20034</v>
+        <v>20104</v>
       </c>
       <c r="F6" s="2">
         <v>39</v>
@@ -795,22 +792,22 @@
         <v>40</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I6" s="5">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="J6" s="5">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="K6" s="6">
         <v>1.32</v>
       </c>
       <c r="L6" s="4">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="M6" s="4">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>16</v>
@@ -818,7 +815,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="B7" s="2">
         <v>162</v>
@@ -827,10 +824,10 @@
         <v>14</v>
       </c>
       <c r="D7" s="4">
-        <v>46176</v>
+        <v>46189</v>
       </c>
       <c r="E7" s="2">
-        <v>20035</v>
+        <v>20105</v>
       </c>
       <c r="F7" s="2">
         <v>39</v>
@@ -839,22 +836,22 @@
         <v>40</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I7" s="5">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="J7" s="5">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="K7" s="6">
         <v>1.32</v>
       </c>
       <c r="L7" s="4">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="M7" s="4">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>16</v>
@@ -862,7 +859,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B8" s="2">
         <v>162</v>
@@ -871,10 +868,10 @@
         <v>14</v>
       </c>
       <c r="D8" s="4">
-        <v>46176</v>
+        <v>46197</v>
       </c>
       <c r="E8" s="2">
-        <v>20082</v>
+        <v>20000</v>
       </c>
       <c r="F8" s="2">
         <v>39</v>
@@ -892,13 +889,13 @@
         <v>3000</v>
       </c>
       <c r="K8" s="6">
-        <v>1.32</v>
+        <v>1.55</v>
       </c>
       <c r="L8" s="4">
-        <v>46268</v>
+        <v>46197</v>
       </c>
       <c r="M8" s="4">
-        <v>46268</v>
+        <v>46197</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>16</v>
@@ -906,7 +903,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B9" s="2">
         <v>162</v>
@@ -915,10 +912,10 @@
         <v>14</v>
       </c>
       <c r="D9" s="4">
-        <v>46176</v>
+        <v>46197</v>
       </c>
       <c r="E9" s="2">
-        <v>20104</v>
+        <v>20011</v>
       </c>
       <c r="F9" s="2">
         <v>39</v>
@@ -927,22 +924,22 @@
         <v>40</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I9" s="5">
-        <v>2000</v>
+        <v>8000</v>
       </c>
       <c r="J9" s="5">
-        <v>2000</v>
+        <v>8000</v>
       </c>
       <c r="K9" s="6">
-        <v>1.32</v>
+        <v>1.55</v>
       </c>
       <c r="L9" s="4">
-        <v>46268</v>
+        <v>46197</v>
       </c>
       <c r="M9" s="4">
-        <v>46268</v>
+        <v>46197</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>16</v>
@@ -950,7 +947,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="B10" s="2">
         <v>162</v>
@@ -959,10 +956,10 @@
         <v>14</v>
       </c>
       <c r="D10" s="4">
-        <v>46177</v>
+        <v>46197</v>
       </c>
       <c r="E10" s="2">
-        <v>14181</v>
+        <v>20012</v>
       </c>
       <c r="F10" s="2">
         <v>39</v>
@@ -971,7 +968,7 @@
         <v>40</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I10" s="5">
         <v>2000</v>
@@ -980,13 +977,13 @@
         <v>2000</v>
       </c>
       <c r="K10" s="6">
-        <v>3.64</v>
+        <v>1.55</v>
       </c>
       <c r="L10" s="4">
-        <v>46269</v>
+        <v>46197</v>
       </c>
       <c r="M10" s="4">
-        <v>46269</v>
+        <v>46197</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>16</v>
@@ -994,7 +991,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B11" s="2">
         <v>162</v>
@@ -1003,7 +1000,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4">
-        <v>46182</v>
+        <v>46197</v>
       </c>
       <c r="E11" s="2">
         <v>20034</v>
@@ -1015,22 +1012,22 @@
         <v>40</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I11" s="5">
-        <v>3000</v>
+        <v>13000</v>
       </c>
       <c r="J11" s="5">
-        <v>3000</v>
+        <v>13000</v>
       </c>
       <c r="K11" s="6">
-        <v>1.32</v>
+        <v>1.88</v>
       </c>
       <c r="L11" s="4">
-        <v>46182</v>
+        <v>46197</v>
       </c>
       <c r="M11" s="4">
-        <v>46274</v>
+        <v>46197</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>16</v>
@@ -1038,7 +1035,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B12" s="2">
         <v>162</v>
@@ -1047,7 +1044,7 @@
         <v>14</v>
       </c>
       <c r="D12" s="4">
-        <v>46182</v>
+        <v>46197</v>
       </c>
       <c r="E12" s="2">
         <v>20035</v>
@@ -1059,22 +1056,22 @@
         <v>40</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I12" s="5">
-        <v>3000</v>
+        <v>10000</v>
       </c>
       <c r="J12" s="5">
-        <v>3000</v>
+        <v>10000</v>
       </c>
       <c r="K12" s="6">
-        <v>1.32</v>
+        <v>1.88</v>
       </c>
       <c r="L12" s="4">
-        <v>46182</v>
+        <v>46197</v>
       </c>
       <c r="M12" s="4">
-        <v>46274</v>
+        <v>46197</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>16</v>
@@ -1082,7 +1079,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B13" s="2">
         <v>162</v>
@@ -1091,10 +1088,10 @@
         <v>14</v>
       </c>
       <c r="D13" s="4">
-        <v>46182</v>
+        <v>46197</v>
       </c>
       <c r="E13" s="2">
-        <v>20104</v>
+        <v>20082</v>
       </c>
       <c r="F13" s="2">
         <v>39</v>
@@ -1103,22 +1100,22 @@
         <v>40</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I13" s="5">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="J13" s="5">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="K13" s="6">
-        <v>1.32</v>
+        <v>1.88</v>
       </c>
       <c r="L13" s="4">
-        <v>46182</v>
+        <v>46197</v>
       </c>
       <c r="M13" s="4">
-        <v>46274</v>
+        <v>46197</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>16</v>
@@ -1126,7 +1123,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B14" s="2">
         <v>162</v>
@@ -1135,10 +1132,10 @@
         <v>14</v>
       </c>
       <c r="D14" s="4">
-        <v>46182</v>
+        <v>46199</v>
       </c>
       <c r="E14" s="2">
-        <v>20106</v>
+        <v>15546</v>
       </c>
       <c r="F14" s="2">
         <v>39</v>
@@ -1147,22 +1144,22 @@
         <v>40</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I14" s="5">
-        <v>1000</v>
+        <v>24000</v>
       </c>
       <c r="J14" s="5">
-        <v>1000</v>
+        <v>24000</v>
       </c>
       <c r="K14" s="6">
-        <v>1.32</v>
+        <v>1.7</v>
       </c>
       <c r="L14" s="4">
-        <v>46182</v>
+        <v>46291</v>
       </c>
       <c r="M14" s="4">
-        <v>46274</v>
+        <v>46291</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>16</v>
@@ -1170,7 +1167,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B15" s="2">
         <v>162</v>
@@ -1179,10 +1176,10 @@
         <v>14</v>
       </c>
       <c r="D15" s="4">
-        <v>46182</v>
+        <v>46204</v>
       </c>
       <c r="E15" s="2">
-        <v>20089</v>
+        <v>20000</v>
       </c>
       <c r="F15" s="2">
         <v>39</v>
@@ -1191,22 +1188,22 @@
         <v>40</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I15" s="5">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="J15" s="5">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="K15" s="6">
-        <v>2.04</v>
+        <v>1.55</v>
       </c>
       <c r="L15" s="4">
-        <v>46182</v>
+        <v>46296</v>
       </c>
       <c r="M15" s="4">
-        <v>46182</v>
+        <v>46296</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>16</v>
@@ -1214,7 +1211,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B16" s="2">
         <v>162</v>
@@ -1223,10 +1220,10 @@
         <v>14</v>
       </c>
       <c r="D16" s="4">
-        <v>46182</v>
+        <v>46204</v>
       </c>
       <c r="E16" s="2">
-        <v>20102</v>
+        <v>20011</v>
       </c>
       <c r="F16" s="2">
         <v>39</v>
@@ -1235,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="I16" s="5">
         <v>3000</v>
@@ -1244,13 +1241,13 @@
         <v>3000</v>
       </c>
       <c r="K16" s="6">
-        <v>2.04</v>
+        <v>1.55</v>
       </c>
       <c r="L16" s="4">
-        <v>46182</v>
+        <v>46296</v>
       </c>
       <c r="M16" s="4">
-        <v>46182</v>
+        <v>46296</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>16</v>
@@ -1258,7 +1255,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B17" s="2">
         <v>162</v>
@@ -1267,7 +1264,7 @@
         <v>14</v>
       </c>
       <c r="D17" s="4">
-        <v>46183</v>
+        <v>46217</v>
       </c>
       <c r="E17" s="2">
         <v>20000</v>
@@ -1279,22 +1276,22 @@
         <v>40</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I17" s="5">
-        <v>7000</v>
+        <v>25000</v>
       </c>
       <c r="J17" s="5">
-        <v>7000</v>
+        <v>25000</v>
       </c>
       <c r="K17" s="6">
-        <v>1.0900000000000001</v>
+        <v>1.55</v>
       </c>
       <c r="L17" s="4">
-        <v>46275</v>
+        <v>46217</v>
       </c>
       <c r="M17" s="4">
-        <v>46275</v>
+        <v>46217</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>16</v>
@@ -1302,7 +1299,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B18" s="2">
         <v>162</v>
@@ -1311,10 +1308,10 @@
         <v>14</v>
       </c>
       <c r="D18" s="4">
-        <v>46183</v>
+        <v>46217</v>
       </c>
       <c r="E18" s="2">
-        <v>20011</v>
+        <v>20002</v>
       </c>
       <c r="F18" s="2">
         <v>39</v>
@@ -1323,7 +1320,7 @@
         <v>40</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I18" s="5">
         <v>3000</v>
@@ -1332,13 +1329,13 @@
         <v>3000</v>
       </c>
       <c r="K18" s="6">
-        <v>1.0900000000000001</v>
+        <v>1.55</v>
       </c>
       <c r="L18" s="4">
-        <v>46275</v>
+        <v>46217</v>
       </c>
       <c r="M18" s="4">
-        <v>46275</v>
+        <v>46217</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>16</v>
@@ -1346,7 +1343,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B19" s="2">
         <v>162</v>
@@ -1355,10 +1352,10 @@
         <v>14</v>
       </c>
       <c r="D19" s="4">
-        <v>46189</v>
+        <v>46217</v>
       </c>
       <c r="E19" s="2">
-        <v>20034</v>
+        <v>20011</v>
       </c>
       <c r="F19" s="2">
         <v>39</v>
@@ -1367,22 +1364,22 @@
         <v>40</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I19" s="5">
-        <v>4000</v>
+        <v>12000</v>
       </c>
       <c r="J19" s="5">
-        <v>4000</v>
+        <v>12000</v>
       </c>
       <c r="K19" s="6">
-        <v>1.32</v>
+        <v>1.55</v>
       </c>
       <c r="L19" s="4">
-        <v>46281</v>
+        <v>46217</v>
       </c>
       <c r="M19" s="4">
-        <v>46281</v>
+        <v>46217</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>16</v>
@@ -1390,7 +1387,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="B20" s="2">
         <v>162</v>
@@ -1399,7 +1396,7 @@
         <v>14</v>
       </c>
       <c r="D20" s="4">
-        <v>46189</v>
+        <v>46232</v>
       </c>
       <c r="E20" s="2">
         <v>20082</v>
@@ -1411,22 +1408,22 @@
         <v>40</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I20" s="5">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="J20" s="5">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="K20" s="6">
-        <v>1.32</v>
+        <v>1.35</v>
       </c>
       <c r="L20" s="4">
-        <v>46281</v>
+        <v>46324</v>
       </c>
       <c r="M20" s="4">
-        <v>46281</v>
+        <v>46324</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>16</v>
@@ -1434,7 +1431,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B21" s="2">
         <v>162</v>
@@ -1443,10 +1440,10 @@
         <v>14</v>
       </c>
       <c r="D21" s="4">
-        <v>46189</v>
+        <v>46239</v>
       </c>
       <c r="E21" s="2">
-        <v>20104</v>
+        <v>14180</v>
       </c>
       <c r="F21" s="2">
         <v>39</v>
@@ -1455,22 +1452,22 @@
         <v>40</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="I21" s="5">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="J21" s="5">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="K21" s="6">
-        <v>1.32</v>
+        <v>5.2</v>
       </c>
       <c r="L21" s="4">
-        <v>46281</v>
+        <v>46331</v>
       </c>
       <c r="M21" s="4">
-        <v>46281</v>
+        <v>46331</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>16</v>
@@ -1478,7 +1475,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="B22" s="2">
         <v>162</v>
@@ -1487,10 +1484,10 @@
         <v>14</v>
       </c>
       <c r="D22" s="4">
-        <v>46189</v>
+        <v>46240</v>
       </c>
       <c r="E22" s="2">
-        <v>20105</v>
+        <v>15546</v>
       </c>
       <c r="F22" s="2">
         <v>39</v>
@@ -1499,22 +1496,22 @@
         <v>40</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="I22" s="5">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="J22" s="5">
-        <v>4000</v>
+        <v>24000</v>
       </c>
       <c r="K22" s="6">
-        <v>1.32</v>
+        <v>1.7</v>
       </c>
       <c r="L22" s="4">
-        <v>46281</v>
+        <v>46326</v>
       </c>
       <c r="M22" s="4">
-        <v>46281</v>
+        <v>46326</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>16</v>
@@ -1522,7 +1519,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B23" s="2">
         <v>162</v>
@@ -1531,10 +1528,10 @@
         <v>14</v>
       </c>
       <c r="D23" s="4">
-        <v>46197</v>
+        <v>46258</v>
       </c>
       <c r="E23" s="2">
-        <v>20000</v>
+        <v>15882</v>
       </c>
       <c r="F23" s="2">
         <v>39</v>
@@ -1542,23 +1539,23 @@
       <c r="G23" s="2">
         <v>40</v>
       </c>
-      <c r="H23" s="3" t="s">
-        <v>26</v>
+      <c r="H23" t="s">
+        <v>28</v>
       </c>
       <c r="I23" s="5">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="J23" s="5">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="K23" s="6">
-        <v>1.55</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="L23" s="4">
-        <v>46197</v>
+        <v>46350</v>
       </c>
       <c r="M23" s="4">
-        <v>46197</v>
+        <v>46350</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>16</v>
@@ -1566,7 +1563,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B24" s="2">
         <v>162</v>
@@ -1575,10 +1572,10 @@
         <v>14</v>
       </c>
       <c r="D24" s="4">
-        <v>46197</v>
+        <v>46259</v>
       </c>
       <c r="E24" s="2">
-        <v>20011</v>
+        <v>17858</v>
       </c>
       <c r="F24" s="2">
         <v>39</v>
@@ -1587,22 +1584,22 @@
         <v>40</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I24" s="5">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="J24" s="5">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="K24" s="6">
-        <v>1.55</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="L24" s="4">
-        <v>46197</v>
+        <v>46350</v>
       </c>
       <c r="M24" s="4">
-        <v>46197</v>
+        <v>46350</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>16</v>
@@ -1610,7 +1607,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="B25" s="2">
         <v>162</v>
@@ -1619,10 +1616,10 @@
         <v>14</v>
       </c>
       <c r="D25" s="4">
-        <v>46197</v>
+        <v>46261</v>
       </c>
       <c r="E25" s="2">
-        <v>20012</v>
+        <v>20102</v>
       </c>
       <c r="F25" s="2">
         <v>39</v>
@@ -1630,8 +1627,8 @@
       <c r="G25" s="2">
         <v>40</v>
       </c>
-      <c r="H25" s="3" t="s">
-        <v>28</v>
+      <c r="H25" t="s">
+        <v>15</v>
       </c>
       <c r="I25" s="5">
         <v>2000</v>
@@ -1640,591 +1637,20 @@
         <v>2000</v>
       </c>
       <c r="K25" s="6">
-        <v>1.55</v>
+        <v>2.97</v>
       </c>
       <c r="L25" s="4">
-        <v>46197</v>
+        <v>46353</v>
       </c>
       <c r="M25" s="4">
-        <v>46197</v>
+        <v>46353</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
-        <v>83</v>
-      </c>
-      <c r="B26" s="2">
-        <v>162</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D26" s="4">
-        <v>46197</v>
-      </c>
-      <c r="E26" s="2">
-        <v>20034</v>
-      </c>
-      <c r="F26" s="2">
-        <v>39</v>
-      </c>
-      <c r="G26" s="2">
-        <v>40</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" s="5">
-        <v>13000</v>
-      </c>
-      <c r="J26" s="5">
-        <v>13000</v>
-      </c>
-      <c r="K26" s="6">
-        <v>1.88</v>
-      </c>
-      <c r="L26" s="4">
-        <v>46197</v>
-      </c>
-      <c r="M26" s="4">
-        <v>46197</v>
-      </c>
-      <c r="N26" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
-        <v>83</v>
-      </c>
-      <c r="B27" s="2">
-        <v>162</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="4">
-        <v>46197</v>
-      </c>
-      <c r="E27" s="2">
-        <v>20035</v>
-      </c>
-      <c r="F27" s="2">
-        <v>39</v>
-      </c>
-      <c r="G27" s="2">
-        <v>40</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I27" s="5">
-        <v>10000</v>
-      </c>
-      <c r="J27" s="5">
-        <v>10000</v>
-      </c>
-      <c r="K27" s="6">
-        <v>1.88</v>
-      </c>
-      <c r="L27" s="4">
-        <v>46197</v>
-      </c>
-      <c r="M27" s="4">
-        <v>46197</v>
-      </c>
-      <c r="N27" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="2">
-        <v>83</v>
-      </c>
-      <c r="B28" s="2">
-        <v>162</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="4">
-        <v>46197</v>
-      </c>
-      <c r="E28" s="2">
-        <v>20082</v>
-      </c>
-      <c r="F28" s="2">
-        <v>39</v>
-      </c>
-      <c r="G28" s="2">
-        <v>40</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28" s="5">
-        <v>4000</v>
-      </c>
-      <c r="J28" s="5">
-        <v>4000</v>
-      </c>
-      <c r="K28" s="6">
-        <v>1.88</v>
-      </c>
-      <c r="L28" s="4">
-        <v>46197</v>
-      </c>
-      <c r="M28" s="4">
-        <v>46197</v>
-      </c>
-      <c r="N28" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="2">
-        <v>84</v>
-      </c>
-      <c r="B29" s="2">
-        <v>162</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" s="4">
-        <v>46199</v>
-      </c>
-      <c r="E29" s="2">
-        <v>15546</v>
-      </c>
-      <c r="F29" s="2">
-        <v>39</v>
-      </c>
-      <c r="G29" s="2">
-        <v>40</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I29" s="5">
-        <v>24000</v>
-      </c>
-      <c r="J29" s="5">
-        <v>24000</v>
-      </c>
-      <c r="K29" s="6">
-        <v>1.7</v>
-      </c>
-      <c r="L29" s="4">
-        <v>46291</v>
-      </c>
-      <c r="M29" s="4">
-        <v>46291</v>
-      </c>
-      <c r="N29" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
-        <v>86</v>
-      </c>
-      <c r="B30" s="2">
-        <v>162</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D30" s="4">
-        <v>46204</v>
-      </c>
-      <c r="E30" s="2">
-        <v>20000</v>
-      </c>
-      <c r="F30" s="2">
-        <v>39</v>
-      </c>
-      <c r="G30" s="2">
-        <v>40</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I30" s="5">
-        <v>5000</v>
-      </c>
-      <c r="J30" s="5">
-        <v>5000</v>
-      </c>
-      <c r="K30" s="6">
-        <v>1.55</v>
-      </c>
-      <c r="L30" s="4">
-        <v>46296</v>
-      </c>
-      <c r="M30" s="4">
-        <v>46296</v>
-      </c>
-      <c r="N30" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="2">
-        <v>86</v>
-      </c>
-      <c r="B31" s="2">
-        <v>162</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D31" s="4">
-        <v>46204</v>
-      </c>
-      <c r="E31" s="2">
-        <v>20011</v>
-      </c>
-      <c r="F31" s="2">
-        <v>39</v>
-      </c>
-      <c r="G31" s="2">
-        <v>40</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I31" s="5">
-        <v>3000</v>
-      </c>
-      <c r="J31" s="5">
-        <v>3000</v>
-      </c>
-      <c r="K31" s="6">
-        <v>1.55</v>
-      </c>
-      <c r="L31" s="4">
-        <v>46296</v>
-      </c>
-      <c r="M31" s="4">
-        <v>46296</v>
-      </c>
-      <c r="N31" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="2">
-        <v>87</v>
-      </c>
-      <c r="B32" s="2">
-        <v>162</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D32" s="4">
-        <v>46217</v>
-      </c>
-      <c r="E32" s="2">
-        <v>20000</v>
-      </c>
-      <c r="F32" s="2">
-        <v>39</v>
-      </c>
-      <c r="G32" s="2">
-        <v>40</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I32" s="5">
-        <v>25000</v>
-      </c>
-      <c r="J32" s="5">
-        <v>25000</v>
-      </c>
-      <c r="K32" s="6">
-        <v>1.55</v>
-      </c>
-      <c r="L32" s="4">
-        <v>46217</v>
-      </c>
-      <c r="M32" s="4">
-        <v>46217</v>
-      </c>
-      <c r="N32" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="2">
-        <v>87</v>
-      </c>
-      <c r="B33" s="2">
-        <v>162</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D33" s="4">
-        <v>46217</v>
-      </c>
-      <c r="E33" s="2">
-        <v>20002</v>
-      </c>
-      <c r="F33" s="2">
-        <v>39</v>
-      </c>
-      <c r="G33" s="2">
-        <v>40</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="I33" s="5">
-        <v>3000</v>
-      </c>
-      <c r="J33" s="5">
-        <v>3000</v>
-      </c>
-      <c r="K33" s="6">
-        <v>1.55</v>
-      </c>
-      <c r="L33" s="4">
-        <v>46217</v>
-      </c>
-      <c r="M33" s="4">
-        <v>46217</v>
-      </c>
-      <c r="N33" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="2">
-        <v>87</v>
-      </c>
-      <c r="B34" s="2">
-        <v>162</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="4">
-        <v>46217</v>
-      </c>
-      <c r="E34" s="2">
-        <v>20011</v>
-      </c>
-      <c r="F34" s="2">
-        <v>39</v>
-      </c>
-      <c r="G34" s="2">
-        <v>40</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I34" s="5">
-        <v>12000</v>
-      </c>
-      <c r="J34" s="5">
-        <v>12000</v>
-      </c>
-      <c r="K34" s="6">
-        <v>1.55</v>
-      </c>
-      <c r="L34" s="4">
-        <v>46217</v>
-      </c>
-      <c r="M34" s="4">
-        <v>46217</v>
-      </c>
-      <c r="N34" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="2">
-        <v>94</v>
-      </c>
-      <c r="B35" s="2">
-        <v>162</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35" s="4">
-        <v>46232</v>
-      </c>
-      <c r="E35" s="2">
-        <v>20082</v>
-      </c>
-      <c r="F35" s="2">
-        <v>39</v>
-      </c>
-      <c r="G35" s="2">
-        <v>40</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I35" s="5">
-        <v>6000</v>
-      </c>
-      <c r="J35" s="5">
-        <v>6000</v>
-      </c>
-      <c r="K35" s="6">
-        <v>1.35</v>
-      </c>
-      <c r="L35" s="4">
-        <v>46324</v>
-      </c>
-      <c r="M35" s="4">
-        <v>46324</v>
-      </c>
-      <c r="N35" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="2">
-        <v>95</v>
-      </c>
-      <c r="B36" s="2">
-        <v>162</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D36" s="4">
-        <v>46239</v>
-      </c>
-      <c r="E36" s="2">
-        <v>14180</v>
-      </c>
-      <c r="F36" s="2">
-        <v>39</v>
-      </c>
-      <c r="G36" s="2">
-        <v>40</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I36" s="5">
-        <v>2000</v>
-      </c>
-      <c r="J36" s="5">
-        <v>2000</v>
-      </c>
-      <c r="K36" s="6">
-        <v>5.2</v>
-      </c>
-      <c r="L36" s="4">
-        <v>46331</v>
-      </c>
-      <c r="M36" s="4">
-        <v>46331</v>
-      </c>
-      <c r="N36" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="2">
-        <v>101</v>
-      </c>
-      <c r="B37" s="2">
-        <v>162</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37" s="4">
-        <v>46240</v>
-      </c>
-      <c r="E37" s="2">
-        <v>15546</v>
-      </c>
-      <c r="F37" s="2">
-        <v>39</v>
-      </c>
-      <c r="G37" s="2">
-        <v>40</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I37" s="5">
-        <v>24000</v>
-      </c>
-      <c r="J37" s="5">
-        <v>24000</v>
-      </c>
-      <c r="K37" s="6">
-        <v>1.7</v>
-      </c>
-      <c r="L37" s="4">
-        <v>46326</v>
-      </c>
-      <c r="M37" s="4">
-        <v>46326</v>
-      </c>
-      <c r="N37" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="2">
-        <v>102</v>
-      </c>
-      <c r="B38" s="2">
-        <v>162</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D38" s="4">
-        <v>46258</v>
-      </c>
-      <c r="E38" s="2">
-        <v>15882</v>
-      </c>
-      <c r="F38" s="2">
-        <v>39</v>
-      </c>
-      <c r="G38" s="2">
-        <v>40</v>
-      </c>
-      <c r="H38" t="s">
-        <v>32</v>
-      </c>
-      <c r="I38" s="5">
-        <v>2000</v>
-      </c>
-      <c r="J38" s="5">
-        <v>2000</v>
-      </c>
-      <c r="K38" s="6">
-        <v>2.12</v>
-      </c>
-      <c r="L38" s="4">
-        <v>46350</v>
-      </c>
-      <c r="M38" s="4">
-        <v>46350</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="9999" orientation="landscape"/>

</xml_diff>

<commit_message>
Atualiza dados do dashboard
</commit_message>
<xml_diff>
--- a/data-source/compras.xlsx
+++ b/data-source/compras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/prompt-smart-stock-sight (4) (1)antig/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="11_A326C178CB385EDFDA183B5B29A248968F540666" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4B0F912-A71B-437D-B77B-F72843E93EEB}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="11_A326C178CB385EDFDA183B5B29A248968F540666" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{456A7303-2961-4E08-BC1B-E6AEA3B06229}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="31">
   <si>
     <t>Núm.OC</t>
   </si>
@@ -113,6 +113,9 @@
   </si>
   <si>
     <t>NAPA METAL LYON PRATA - PU 0.9MM</t>
+  </si>
+  <si>
+    <t>NAPA METAL CHARM PRATA - PU 0.9MM</t>
   </si>
 </sst>
 </file>
@@ -530,23 +533,23 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
-    <col min="2" max="2" width="5.44140625" customWidth="1"/>
-    <col min="3" max="3" width="36.44140625" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" customWidth="1"/>
-    <col min="8" max="8" width="43" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="12.21875" customWidth="1"/>
-    <col min="11" max="11" width="7.77734375" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" customWidth="1"/>
-    <col min="13" max="13" width="13.6640625" customWidth="1"/>
-    <col min="14" max="14" width="9" customWidth="1"/>
+    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -1646,6 +1649,252 @@
         <v>46353</v>
       </c>
       <c r="N25" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>103</v>
+      </c>
+      <c r="B26" s="2">
+        <v>162</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="4">
+        <v>46262</v>
+      </c>
+      <c r="E26" s="2">
+        <v>20011</v>
+      </c>
+      <c r="F26" s="2">
+        <v>39</v>
+      </c>
+      <c r="G26" s="2">
+        <v>40</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I26" s="5">
+        <v>5000</v>
+      </c>
+      <c r="J26" s="5">
+        <v>5000</v>
+      </c>
+      <c r="L26" s="4">
+        <v>46354</v>
+      </c>
+      <c r="M26" s="4">
+        <v>46354</v>
+      </c>
+      <c r="N26" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>103</v>
+      </c>
+      <c r="B27" s="2">
+        <v>162</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="4">
+        <v>46263</v>
+      </c>
+      <c r="E27" s="2">
+        <v>20104</v>
+      </c>
+      <c r="F27" s="2">
+        <v>39</v>
+      </c>
+      <c r="G27" s="2">
+        <v>40</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="5">
+        <v>5000</v>
+      </c>
+      <c r="J27" s="5">
+        <v>5000</v>
+      </c>
+      <c r="L27" s="4">
+        <v>46355</v>
+      </c>
+      <c r="M27" s="4">
+        <v>46355</v>
+      </c>
+      <c r="N27" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>103</v>
+      </c>
+      <c r="B28" s="2">
+        <v>162</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="4">
+        <v>46264</v>
+      </c>
+      <c r="E28" s="2">
+        <v>20105</v>
+      </c>
+      <c r="F28" s="2">
+        <v>39</v>
+      </c>
+      <c r="G28" s="2">
+        <v>40</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="5">
+        <v>2000</v>
+      </c>
+      <c r="J28" s="5">
+        <v>2000</v>
+      </c>
+      <c r="L28" s="4">
+        <v>46356</v>
+      </c>
+      <c r="M28" s="4">
+        <v>46356</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>103</v>
+      </c>
+      <c r="B29" s="2">
+        <v>162</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="4">
+        <v>46265</v>
+      </c>
+      <c r="E29" s="2">
+        <v>15882</v>
+      </c>
+      <c r="F29" s="2">
+        <v>39</v>
+      </c>
+      <c r="G29" s="2">
+        <v>40</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I29" s="5">
+        <v>3000</v>
+      </c>
+      <c r="J29" s="5">
+        <v>3000</v>
+      </c>
+      <c r="L29" s="4">
+        <v>46357</v>
+      </c>
+      <c r="M29" s="4">
+        <v>46357</v>
+      </c>
+      <c r="N29" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>103</v>
+      </c>
+      <c r="B30" s="2">
+        <v>162</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="4">
+        <v>46266</v>
+      </c>
+      <c r="E30" s="2">
+        <v>20102</v>
+      </c>
+      <c r="F30" s="2">
+        <v>39</v>
+      </c>
+      <c r="G30" s="2">
+        <v>40</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I30" s="5">
+        <v>1000</v>
+      </c>
+      <c r="J30" s="5">
+        <v>1000</v>
+      </c>
+      <c r="L30" s="4">
+        <v>46358</v>
+      </c>
+      <c r="M30" s="4">
+        <v>46358</v>
+      </c>
+      <c r="N30" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>103</v>
+      </c>
+      <c r="B31" s="2">
+        <v>162</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="4">
+        <v>46267</v>
+      </c>
+      <c r="E31" s="2">
+        <v>20103</v>
+      </c>
+      <c r="F31" s="2">
+        <v>39</v>
+      </c>
+      <c r="G31" s="2">
+        <v>40</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I31" s="5">
+        <v>2000</v>
+      </c>
+      <c r="J31" s="5">
+        <v>2000</v>
+      </c>
+      <c r="L31" s="4">
+        <v>46359</v>
+      </c>
+      <c r="M31" s="4">
+        <v>46359</v>
+      </c>
+      <c r="N31" s="3" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>